<commit_message>
Refactored crop rules into modules. Added crop family alerts.
</commit_message>
<xml_diff>
--- a/data/Garden_Planning.xlsx
+++ b/data/Garden_Planning.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wcwil\OneDrive\Documents\Python Projects\garden_app\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wcwil\OneDrive\Documents\Python Projects\garden_app\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A7FEF9B-EC7B-4CF1-886C-84CCC43ECC6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F585EC63-6294-4CBE-9E70-E5902EBE1B97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3555" yWindow="0" windowWidth="26595" windowHeight="20880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2010" yWindow="330" windowWidth="26595" windowHeight="20880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CropDatabase" sheetId="2" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Helper Lists" sheetId="3" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CropDatabase!$A$2:$I$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CropDatabase!$B$2:$K$2</definedName>
     <definedName name="Deep_Raised_Bed" localSheetId="1">'2026'!$D$52:$F$62</definedName>
     <definedName name="Deep_Raised_Bed">'Diagram Template'!$D$52:$F$62</definedName>
     <definedName name="DRB" localSheetId="1">'2026'!$D$52:$F$62</definedName>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="728" uniqueCount="248">
   <si>
     <t>Spring</t>
   </si>
@@ -329,9 +329,6 @@
     <t>Cf</t>
   </si>
   <si>
-    <t>HIgh</t>
-  </si>
-  <si>
     <t>Celery</t>
   </si>
   <si>
@@ -753,6 +750,51 @@
   </si>
   <si>
     <t>Fence</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Legume</t>
+  </si>
+  <si>
+    <t>N-Fixing</t>
+  </si>
+  <si>
+    <t>N-Fixing / Cover Crop</t>
+  </si>
+  <si>
+    <t>Crop Family</t>
+  </si>
+  <si>
+    <t>Leafy Green</t>
+  </si>
+  <si>
+    <t>Herb</t>
+  </si>
+  <si>
+    <t>Root</t>
+  </si>
+  <si>
+    <t>Solanaceae</t>
+  </si>
+  <si>
+    <t>Brassica</t>
+  </si>
+  <si>
+    <t>Allium</t>
+  </si>
+  <si>
+    <t>Cucurbit</t>
+  </si>
+  <si>
+    <t>Apiaceae</t>
+  </si>
+  <si>
+    <t>Grass</t>
   </si>
 </sst>
 </file>
@@ -1213,7 +1255,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
@@ -1371,6 +1413,12 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1768,8 +1816,11 @@
       <c r="I2" s="67" t="s">
         <v>30</v>
       </c>
-      <c r="J2" s="68" t="s">
+      <c r="J2" s="67" t="s">
         <v>31</v>
+      </c>
+      <c r="K2" s="67" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
@@ -1800,6 +1851,15 @@
       <c r="I3" t="s">
         <v>40</v>
       </c>
+      <c r="J3" t="s">
+        <v>233</v>
+      </c>
+      <c r="K3" s="71" t="s">
+        <v>239</v>
+      </c>
+      <c r="L3" s="70"/>
+      <c r="M3" s="70"/>
+      <c r="N3" s="71"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="64" t="s">
@@ -1829,6 +1889,15 @@
       <c r="I4" t="s">
         <v>40</v>
       </c>
+      <c r="J4" t="s">
+        <v>233</v>
+      </c>
+      <c r="K4" s="71" t="s">
+        <v>239</v>
+      </c>
+      <c r="L4" s="71"/>
+      <c r="M4" s="71"/>
+      <c r="N4" s="71"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="64" t="s">
@@ -1858,6 +1927,15 @@
       <c r="I5" t="s">
         <v>52</v>
       </c>
+      <c r="J5" t="s">
+        <v>233</v>
+      </c>
+      <c r="K5" s="71" t="s">
+        <v>240</v>
+      </c>
+      <c r="L5" s="71"/>
+      <c r="M5" s="71"/>
+      <c r="N5" s="71"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="64" t="s">
@@ -1887,6 +1965,15 @@
       <c r="I6" t="s">
         <v>58</v>
       </c>
+      <c r="J6" t="s">
+        <v>234</v>
+      </c>
+      <c r="K6" s="71" t="s">
+        <v>241</v>
+      </c>
+      <c r="L6" s="71"/>
+      <c r="M6" s="71"/>
+      <c r="N6" s="71"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="64" t="s">
@@ -1916,6 +2003,15 @@
       <c r="I7" t="s">
         <v>52</v>
       </c>
+      <c r="J7" t="s">
+        <v>233</v>
+      </c>
+      <c r="K7" s="71" t="s">
+        <v>242</v>
+      </c>
+      <c r="L7" s="71"/>
+      <c r="M7" s="71"/>
+      <c r="N7" s="71"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="64" t="s">
@@ -1948,6 +2044,12 @@
       <c r="J8" t="s">
         <v>67</v>
       </c>
+      <c r="K8" s="71" t="s">
+        <v>243</v>
+      </c>
+      <c r="L8" s="71"/>
+      <c r="M8" s="71"/>
+      <c r="N8" s="71"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="64" t="s">
@@ -1977,6 +2079,15 @@
       <c r="I9" t="s">
         <v>40</v>
       </c>
+      <c r="J9" t="s">
+        <v>67</v>
+      </c>
+      <c r="K9" s="71" t="s">
+        <v>243</v>
+      </c>
+      <c r="L9" s="71"/>
+      <c r="M9" s="71"/>
+      <c r="N9" s="71"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="64" t="s">
@@ -2006,6 +2117,15 @@
       <c r="I10" t="s">
         <v>40</v>
       </c>
+      <c r="J10" t="s">
+        <v>233</v>
+      </c>
+      <c r="K10" s="71" t="s">
+        <v>244</v>
+      </c>
+      <c r="L10" s="71"/>
+      <c r="M10" s="71"/>
+      <c r="N10" s="71"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="64" t="s">
@@ -2035,6 +2155,15 @@
       <c r="I11" t="s">
         <v>52</v>
       </c>
+      <c r="J11" t="s">
+        <v>236</v>
+      </c>
+      <c r="K11" s="71" t="s">
+        <v>235</v>
+      </c>
+      <c r="L11" s="71"/>
+      <c r="M11" s="71"/>
+      <c r="N11" s="71"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="64" t="s">
@@ -2064,6 +2193,15 @@
       <c r="I12" t="s">
         <v>52</v>
       </c>
+      <c r="J12" t="s">
+        <v>67</v>
+      </c>
+      <c r="K12" s="71" t="s">
+        <v>245</v>
+      </c>
+      <c r="L12" s="71"/>
+      <c r="M12" s="71"/>
+      <c r="N12" s="71"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="64" t="s">
@@ -2093,6 +2231,15 @@
       <c r="I13" t="s">
         <v>58</v>
       </c>
+      <c r="J13" t="s">
+        <v>67</v>
+      </c>
+      <c r="K13" s="71" t="s">
+        <v>243</v>
+      </c>
+      <c r="L13" s="71"/>
+      <c r="M13" s="71"/>
+      <c r="N13" s="71"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="64" t="s">
@@ -2122,6 +2269,15 @@
       <c r="I14" t="s">
         <v>58</v>
       </c>
+      <c r="J14" t="s">
+        <v>234</v>
+      </c>
+      <c r="K14" s="71" t="s">
+        <v>241</v>
+      </c>
+      <c r="L14" s="71"/>
+      <c r="M14" s="71"/>
+      <c r="N14" s="71"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="64" t="s">
@@ -2152,15 +2308,21 @@
         <v>58</v>
       </c>
       <c r="J15" t="s">
-        <v>92</v>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="K15" s="71" t="s">
+        <v>243</v>
+      </c>
+      <c r="L15" s="71"/>
+      <c r="M15" s="71"/>
+      <c r="N15" s="71"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="64" t="s">
+        <v>92</v>
+      </c>
+      <c r="B16" t="s">
         <v>93</v>
-      </c>
-      <c r="B16" t="s">
-        <v>94</v>
       </c>
       <c r="C16" t="s">
         <v>34</v>
@@ -2169,16 +2331,16 @@
         <v>48</v>
       </c>
       <c r="E16" t="s">
+        <v>94</v>
+      </c>
+      <c r="F16" t="s">
         <v>95</v>
-      </c>
-      <c r="F16" t="s">
-        <v>96</v>
       </c>
       <c r="G16" t="s">
         <v>62</v>
       </c>
       <c r="H16" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I16" t="s">
         <v>58</v>
@@ -2186,42 +2348,57 @@
       <c r="J16" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K16" s="71" t="s">
+        <v>246</v>
+      </c>
+      <c r="L16" s="71"/>
+      <c r="M16" s="71"/>
+      <c r="N16" s="71"/>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="64" t="s">
+        <v>97</v>
+      </c>
+      <c r="B17" t="s">
         <v>98</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>99</v>
-      </c>
-      <c r="C17" t="s">
-        <v>100</v>
       </c>
       <c r="D17" t="s">
         <v>35</v>
       </c>
       <c r="E17" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F17" t="s">
         <v>49</v>
       </c>
       <c r="G17" t="s">
+        <v>101</v>
+      </c>
+      <c r="H17" t="s">
         <v>102</v>
-      </c>
-      <c r="H17" t="s">
-        <v>103</v>
       </c>
       <c r="I17" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J17" t="s">
+        <v>234</v>
+      </c>
+      <c r="K17" s="71" t="s">
+        <v>240</v>
+      </c>
+      <c r="L17" s="71"/>
+      <c r="M17" s="71"/>
+      <c r="N17" s="71"/>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="64" t="s">
+        <v>103</v>
+      </c>
+      <c r="B18" t="s">
         <v>104</v>
-      </c>
-      <c r="B18" t="s">
-        <v>105</v>
       </c>
       <c r="C18" t="s">
         <v>34</v>
@@ -2230,27 +2407,36 @@
         <v>35</v>
       </c>
       <c r="E18" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F18" t="s">
         <v>61</v>
       </c>
       <c r="G18" t="s">
+        <v>106</v>
+      </c>
+      <c r="H18" t="s">
         <v>107</v>
-      </c>
-      <c r="H18" t="s">
-        <v>108</v>
       </c>
       <c r="I18" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J18" t="s">
+        <v>234</v>
+      </c>
+      <c r="K18" s="71" t="s">
+        <v>244</v>
+      </c>
+      <c r="L18" s="71"/>
+      <c r="M18" s="71"/>
+      <c r="N18" s="71"/>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="64" t="s">
+        <v>108</v>
+      </c>
+      <c r="B19" t="s">
         <v>109</v>
-      </c>
-      <c r="B19" t="s">
-        <v>110</v>
       </c>
       <c r="C19" t="s">
         <v>34</v>
@@ -2262,7 +2448,7 @@
         <v>36</v>
       </c>
       <c r="F19" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G19" t="s">
         <v>66</v>
@@ -2273,42 +2459,60 @@
       <c r="I19" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J19" t="s">
+        <v>234</v>
+      </c>
+      <c r="K19" s="71" t="s">
+        <v>240</v>
+      </c>
+      <c r="L19" s="71"/>
+      <c r="M19" s="71"/>
+      <c r="N19" s="71"/>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="64" t="s">
+        <v>111</v>
+      </c>
+      <c r="B20" t="s">
         <v>112</v>
       </c>
-      <c r="B20" t="s">
-        <v>113</v>
-      </c>
       <c r="C20" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D20" t="s">
         <v>35</v>
       </c>
       <c r="E20" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F20" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G20" t="s">
         <v>50</v>
       </c>
       <c r="H20" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I20" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J20" t="s">
+        <v>234</v>
+      </c>
+      <c r="K20" s="71" t="s">
+        <v>99</v>
+      </c>
+      <c r="L20" s="71"/>
+      <c r="M20" s="71"/>
+      <c r="N20" s="71"/>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" s="64" t="s">
+        <v>114</v>
+      </c>
+      <c r="B21" t="s">
         <v>115</v>
-      </c>
-      <c r="B21" t="s">
-        <v>116</v>
       </c>
       <c r="C21" t="s">
         <v>34</v>
@@ -2320,13 +2524,13 @@
         <v>1</v>
       </c>
       <c r="F21" t="s">
+        <v>116</v>
+      </c>
+      <c r="G21" t="s">
         <v>117</v>
       </c>
-      <c r="G21" t="s">
+      <c r="H21" t="s">
         <v>118</v>
-      </c>
-      <c r="H21" t="s">
-        <v>119</v>
       </c>
       <c r="I21" t="s">
         <v>52</v>
@@ -2334,42 +2538,57 @@
       <c r="J21" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K21" s="71" t="s">
+        <v>247</v>
+      </c>
+      <c r="L21" s="71"/>
+      <c r="M21" s="71"/>
+      <c r="N21" s="71"/>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="64" t="s">
+        <v>119</v>
+      </c>
+      <c r="B22" t="s">
         <v>120</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
         <v>121</v>
-      </c>
-      <c r="C22" t="s">
-        <v>122</v>
       </c>
       <c r="D22" t="s">
         <v>35</v>
       </c>
       <c r="E22" t="s">
+        <v>122</v>
+      </c>
+      <c r="F22" t="s">
         <v>123</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>124</v>
       </c>
-      <c r="G22" t="s">
+      <c r="H22" t="s">
         <v>125</v>
-      </c>
-      <c r="H22" t="s">
-        <v>126</v>
       </c>
       <c r="I22" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J22" t="s">
+        <v>236</v>
+      </c>
+      <c r="K22" s="71" t="s">
+        <v>235</v>
+      </c>
+      <c r="L22" s="71"/>
+      <c r="M22" s="71"/>
+      <c r="N22" s="71"/>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="64" t="s">
+        <v>126</v>
+      </c>
+      <c r="B23" t="s">
         <v>127</v>
-      </c>
-      <c r="B23" t="s">
-        <v>128</v>
       </c>
       <c r="C23" t="s">
         <v>34</v>
@@ -2381,24 +2600,33 @@
         <v>1</v>
       </c>
       <c r="F23" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G23" t="s">
         <v>50</v>
       </c>
       <c r="H23" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I23" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J23" t="s">
+        <v>233</v>
+      </c>
+      <c r="K23" s="71" t="s">
+        <v>245</v>
+      </c>
+      <c r="L23" s="71"/>
+      <c r="M23" s="71"/>
+      <c r="N23" s="71"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="64" t="s">
+        <v>130</v>
+      </c>
+      <c r="B24" t="s">
         <v>131</v>
-      </c>
-      <c r="B24" t="s">
-        <v>132</v>
       </c>
       <c r="C24" t="s">
         <v>34</v>
@@ -2407,13 +2635,13 @@
         <v>35</v>
       </c>
       <c r="E24" t="s">
+        <v>100</v>
+      </c>
+      <c r="F24" t="s">
+        <v>128</v>
+      </c>
+      <c r="G24" t="s">
         <v>101</v>
-      </c>
-      <c r="F24" t="s">
-        <v>129</v>
-      </c>
-      <c r="G24" t="s">
-        <v>102</v>
       </c>
       <c r="H24" t="s">
         <v>39</v>
@@ -2421,42 +2649,60 @@
       <c r="I24" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J24" t="s">
+        <v>234</v>
+      </c>
+      <c r="K24" s="71" t="s">
+        <v>240</v>
+      </c>
+      <c r="L24" s="71"/>
+      <c r="M24" s="71"/>
+      <c r="N24" s="71"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="64" t="s">
+        <v>132</v>
+      </c>
+      <c r="B25" t="s">
         <v>133</v>
       </c>
-      <c r="B25" t="s">
-        <v>134</v>
-      </c>
       <c r="C25" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D25" t="s">
         <v>35</v>
       </c>
       <c r="E25" t="s">
+        <v>122</v>
+      </c>
+      <c r="F25" t="s">
         <v>123</v>
       </c>
-      <c r="F25" t="s">
-        <v>124</v>
-      </c>
       <c r="G25" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H25" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I25" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J25" t="s">
+        <v>237</v>
+      </c>
+      <c r="K25" s="71" t="s">
+        <v>121</v>
+      </c>
+      <c r="L25" s="71"/>
+      <c r="M25" s="71"/>
+      <c r="N25" s="71"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="64" t="s">
+        <v>135</v>
+      </c>
+      <c r="B26" t="s">
         <v>136</v>
-      </c>
-      <c r="B26" t="s">
-        <v>137</v>
       </c>
       <c r="C26" t="s">
         <v>34</v>
@@ -2465,13 +2711,13 @@
         <v>35</v>
       </c>
       <c r="E26" t="s">
+        <v>137</v>
+      </c>
+      <c r="F26" t="s">
         <v>138</v>
       </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
         <v>139</v>
-      </c>
-      <c r="G26" t="s">
-        <v>140</v>
       </c>
       <c r="H26" t="s">
         <v>57</v>
@@ -2479,13 +2725,22 @@
       <c r="I26" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J26" t="s">
+        <v>233</v>
+      </c>
+      <c r="K26" s="71" t="s">
+        <v>244</v>
+      </c>
+      <c r="L26" s="71"/>
+      <c r="M26" s="71"/>
+      <c r="N26" s="71"/>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="64" t="s">
+        <v>140</v>
+      </c>
+      <c r="B27" t="s">
         <v>141</v>
-      </c>
-      <c r="B27" t="s">
-        <v>142</v>
       </c>
       <c r="C27" t="s">
         <v>34</v>
@@ -2508,16 +2763,25 @@
       <c r="I27" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J27" t="s">
+        <v>233</v>
+      </c>
+      <c r="K27" s="71" t="s">
+        <v>244</v>
+      </c>
+      <c r="L27" s="71"/>
+      <c r="M27" s="71"/>
+      <c r="N27" s="71"/>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="64" t="s">
+        <v>142</v>
+      </c>
+      <c r="B28" t="s">
         <v>143</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
         <v>144</v>
-      </c>
-      <c r="C28" t="s">
-        <v>145</v>
       </c>
       <c r="D28" t="s">
         <v>48</v>
@@ -2529,21 +2793,30 @@
         <v>49</v>
       </c>
       <c r="G28" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H28" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I28" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J28" t="s">
+        <v>67</v>
+      </c>
+      <c r="K28" s="71" t="s">
+        <v>245</v>
+      </c>
+      <c r="L28" s="71"/>
+      <c r="M28" s="71"/>
+      <c r="N28" s="71"/>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="64" t="s">
+        <v>146</v>
+      </c>
+      <c r="B29" t="s">
         <v>147</v>
-      </c>
-      <c r="B29" t="s">
-        <v>148</v>
       </c>
       <c r="C29" t="s">
         <v>34</v>
@@ -2566,13 +2839,22 @@
       <c r="I29" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J29" t="s">
+        <v>233</v>
+      </c>
+      <c r="K29" s="71" t="s">
+        <v>242</v>
+      </c>
+      <c r="L29" s="71"/>
+      <c r="M29" s="71"/>
+      <c r="N29" s="71"/>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="64" t="s">
+        <v>148</v>
+      </c>
+      <c r="B30" t="s">
         <v>149</v>
-      </c>
-      <c r="B30" t="s">
-        <v>150</v>
       </c>
       <c r="C30" t="s">
         <v>34</v>
@@ -2584,10 +2866,10 @@
         <v>70</v>
       </c>
       <c r="F30" t="s">
+        <v>150</v>
+      </c>
+      <c r="G30" t="s">
         <v>151</v>
-      </c>
-      <c r="G30" t="s">
-        <v>152</v>
       </c>
       <c r="H30" t="s">
         <v>57</v>
@@ -2595,57 +2877,75 @@
       <c r="I30" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J30" t="s">
+        <v>67</v>
+      </c>
+      <c r="K30" s="71" t="s">
+        <v>243</v>
+      </c>
+      <c r="L30" s="71"/>
+      <c r="M30" s="71"/>
+      <c r="N30" s="71"/>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="64" t="s">
+        <v>152</v>
+      </c>
+      <c r="B31" t="s">
         <v>153</v>
       </c>
-      <c r="B31" t="s">
-        <v>154</v>
-      </c>
       <c r="C31" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D31" t="s">
         <v>35</v>
       </c>
       <c r="E31" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F31" t="s">
         <v>61</v>
       </c>
       <c r="G31" t="s">
+        <v>101</v>
+      </c>
+      <c r="H31" t="s">
         <v>102</v>
-      </c>
-      <c r="H31" t="s">
-        <v>103</v>
       </c>
       <c r="I31" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J31" t="s">
+        <v>234</v>
+      </c>
+      <c r="K31" s="71" t="s">
+        <v>240</v>
+      </c>
+      <c r="L31" s="71"/>
+      <c r="M31" s="71"/>
+      <c r="N31" s="71"/>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="64" t="s">
+        <v>154</v>
+      </c>
+      <c r="B32" t="s">
         <v>155</v>
-      </c>
-      <c r="B32" t="s">
-        <v>156</v>
       </c>
       <c r="C32" t="s">
         <v>34</v>
       </c>
       <c r="D32" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E32" t="s">
         <v>36</v>
       </c>
       <c r="F32" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G32" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H32" t="s">
         <v>76</v>
@@ -2653,16 +2953,25 @@
       <c r="I32" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J32" t="s">
+        <v>233</v>
+      </c>
+      <c r="K32" s="71" t="s">
+        <v>239</v>
+      </c>
+      <c r="L32" s="71"/>
+      <c r="M32" s="71"/>
+      <c r="N32" s="71"/>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="64" t="s">
+        <v>158</v>
+      </c>
+      <c r="B33" t="s">
         <v>159</v>
       </c>
-      <c r="B33" t="s">
-        <v>160</v>
-      </c>
       <c r="C33" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D33" t="s">
         <v>48</v>
@@ -2677,21 +2986,30 @@
         <v>82</v>
       </c>
       <c r="H33" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I33" t="s">
+        <v>160</v>
+      </c>
+      <c r="J33" t="s">
+        <v>67</v>
+      </c>
+      <c r="K33" s="71" t="s">
+        <v>245</v>
+      </c>
+      <c r="L33" s="71"/>
+      <c r="M33" s="71"/>
+      <c r="N33" s="71"/>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A34" s="64" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="64" t="s">
+      <c r="B34" t="s">
         <v>162</v>
       </c>
-      <c r="B34" t="s">
-        <v>163</v>
-      </c>
       <c r="C34" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D34" t="s">
         <v>35</v>
@@ -2703,50 +3021,68 @@
         <v>49</v>
       </c>
       <c r="G34" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H34" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I34" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J34" t="s">
+        <v>236</v>
+      </c>
+      <c r="K34" s="71" t="s">
+        <v>235</v>
+      </c>
+      <c r="L34" s="71"/>
+      <c r="M34" s="71"/>
+      <c r="N34" s="71"/>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="64" t="s">
+        <v>163</v>
+      </c>
+      <c r="B35" t="s">
         <v>164</v>
       </c>
-      <c r="B35" t="s">
-        <v>165</v>
-      </c>
       <c r="C35" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D35" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E35" t="s">
         <v>1</v>
       </c>
       <c r="F35" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G35" t="s">
         <v>56</v>
       </c>
       <c r="H35" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I35" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J35" t="s">
+        <v>234</v>
+      </c>
+      <c r="K35" s="71" t="s">
+        <v>99</v>
+      </c>
+      <c r="L35" s="71"/>
+      <c r="M35" s="71"/>
+      <c r="N35" s="71"/>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="64" t="s">
+        <v>166</v>
+      </c>
+      <c r="B36" t="s">
         <v>167</v>
-      </c>
-      <c r="B36" t="s">
-        <v>168</v>
       </c>
       <c r="C36" t="s">
         <v>34</v>
@@ -2769,13 +3105,22 @@
       <c r="I36" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J36" t="s">
+        <v>233</v>
+      </c>
+      <c r="K36" s="71" t="s">
+        <v>239</v>
+      </c>
+      <c r="L36" s="71"/>
+      <c r="M36" s="71"/>
+      <c r="N36" s="71"/>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="64" t="s">
+        <v>168</v>
+      </c>
+      <c r="B37" t="s">
         <v>169</v>
-      </c>
-      <c r="B37" t="s">
-        <v>170</v>
       </c>
       <c r="C37" t="s">
         <v>34</v>
@@ -2784,27 +3129,36 @@
         <v>48</v>
       </c>
       <c r="E37" t="s">
+        <v>170</v>
+      </c>
+      <c r="F37" t="s">
         <v>171</v>
       </c>
-      <c r="F37" t="s">
+      <c r="G37" t="s">
         <v>172</v>
       </c>
-      <c r="G37" t="s">
+      <c r="H37" t="s">
         <v>173</v>
       </c>
-      <c r="H37" t="s">
+      <c r="I37" t="s">
         <v>174</v>
       </c>
-      <c r="I37" t="s">
+      <c r="J37" t="s">
+        <v>234</v>
+      </c>
+      <c r="K37" s="71" t="s">
+        <v>239</v>
+      </c>
+      <c r="L37" s="71"/>
+      <c r="M37" s="71"/>
+      <c r="N37" s="71"/>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A38" s="64" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="64" t="s">
+      <c r="B38" t="s">
         <v>176</v>
-      </c>
-      <c r="B38" t="s">
-        <v>177</v>
       </c>
       <c r="C38" t="s">
         <v>34</v>
@@ -2813,7 +3167,7 @@
         <v>48</v>
       </c>
       <c r="E38" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F38" t="s">
         <v>61</v>
@@ -2827,19 +3181,28 @@
       <c r="I38" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J38" t="s">
+        <v>234</v>
+      </c>
+      <c r="K38" s="71" t="s">
+        <v>240</v>
+      </c>
+      <c r="L38" s="71"/>
+      <c r="M38" s="71"/>
+      <c r="N38" s="71"/>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" s="64" t="s">
+        <v>177</v>
+      </c>
+      <c r="B39" t="s">
         <v>178</v>
-      </c>
-      <c r="B39" t="s">
-        <v>179</v>
       </c>
       <c r="C39" t="s">
         <v>34</v>
       </c>
       <c r="D39" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E39" t="s">
         <v>74</v>
@@ -2856,13 +3219,22 @@
       <c r="I39" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J39" t="s">
+        <v>234</v>
+      </c>
+      <c r="K39" s="71" t="s">
+        <v>240</v>
+      </c>
+      <c r="L39" s="71"/>
+      <c r="M39" s="71"/>
+      <c r="N39" s="71"/>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" s="64" t="s">
+        <v>179</v>
+      </c>
+      <c r="B40" t="s">
         <v>180</v>
-      </c>
-      <c r="B40" t="s">
-        <v>181</v>
       </c>
       <c r="C40" t="s">
         <v>34</v>
@@ -2871,27 +3243,36 @@
         <v>35</v>
       </c>
       <c r="E40" t="s">
+        <v>181</v>
+      </c>
+      <c r="F40" t="s">
+        <v>128</v>
+      </c>
+      <c r="G40" t="s">
         <v>182</v>
       </c>
-      <c r="F40" t="s">
-        <v>129</v>
-      </c>
-      <c r="G40" t="s">
+      <c r="H40" t="s">
         <v>183</v>
-      </c>
-      <c r="H40" t="s">
-        <v>184</v>
       </c>
       <c r="I40" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J40" t="s">
+        <v>234</v>
+      </c>
+      <c r="K40" s="71" t="s">
+        <v>241</v>
+      </c>
+      <c r="L40" s="71"/>
+      <c r="M40" s="71"/>
+      <c r="N40" s="71"/>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" s="64" t="s">
+        <v>184</v>
+      </c>
+      <c r="B41" t="s">
         <v>185</v>
-      </c>
-      <c r="B41" t="s">
-        <v>186</v>
       </c>
       <c r="C41" t="s">
         <v>34</v>
@@ -2903,24 +3284,33 @@
         <v>1</v>
       </c>
       <c r="F41" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G41" t="s">
         <v>82</v>
       </c>
       <c r="H41" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I41" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J41" t="s">
+        <v>67</v>
+      </c>
+      <c r="K41" s="71" t="s">
+        <v>245</v>
+      </c>
+      <c r="L41" s="71"/>
+      <c r="M41" s="71"/>
+      <c r="N41" s="71"/>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" s="64" t="s">
+        <v>187</v>
+      </c>
+      <c r="B42" t="s">
         <v>188</v>
-      </c>
-      <c r="B42" t="s">
-        <v>189</v>
       </c>
       <c r="C42" t="s">
         <v>34</v>
@@ -2935,21 +3325,30 @@
         <v>43</v>
       </c>
       <c r="G42" t="s">
+        <v>189</v>
+      </c>
+      <c r="H42" t="s">
         <v>190</v>
-      </c>
-      <c r="H42" t="s">
-        <v>191</v>
       </c>
       <c r="I42" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J42" t="s">
+        <v>234</v>
+      </c>
+      <c r="K42" s="71" t="s">
+        <v>241</v>
+      </c>
+      <c r="L42" s="71"/>
+      <c r="M42" s="71"/>
+      <c r="N42" s="71"/>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" s="64" t="s">
+        <v>191</v>
+      </c>
+      <c r="B43" t="s">
         <v>192</v>
-      </c>
-      <c r="B43" t="s">
-        <v>193</v>
       </c>
       <c r="C43" t="s">
         <v>34</v>
@@ -2958,13 +3357,13 @@
         <v>48</v>
       </c>
       <c r="E43" t="s">
+        <v>193</v>
+      </c>
+      <c r="F43" t="s">
         <v>194</v>
       </c>
-      <c r="F43" t="s">
+      <c r="G43" t="s">
         <v>195</v>
-      </c>
-      <c r="G43" t="s">
-        <v>196</v>
       </c>
       <c r="H43" t="s">
         <v>39</v>
@@ -2972,13 +3371,22 @@
       <c r="I43" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J43" t="s">
+        <v>233</v>
+      </c>
+      <c r="K43" s="71" t="s">
+        <v>244</v>
+      </c>
+      <c r="L43" s="71"/>
+      <c r="M43" s="71"/>
+      <c r="N43" s="71"/>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" s="64" t="s">
+        <v>196</v>
+      </c>
+      <c r="B44" t="s">
         <v>197</v>
-      </c>
-      <c r="B44" t="s">
-        <v>198</v>
       </c>
       <c r="C44" t="s">
         <v>34</v>
@@ -2987,13 +3395,13 @@
         <v>35</v>
       </c>
       <c r="E44" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F44" t="s">
         <v>49</v>
       </c>
       <c r="G44" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="H44" t="s">
         <v>51</v>
@@ -3001,13 +3409,22 @@
       <c r="I44" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J44" t="s">
+        <v>234</v>
+      </c>
+      <c r="K44" s="71" t="s">
+        <v>240</v>
+      </c>
+      <c r="L44" s="71"/>
+      <c r="M44" s="71"/>
+      <c r="N44" s="71"/>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" s="64" t="s">
+        <v>198</v>
+      </c>
+      <c r="B45" t="s">
         <v>199</v>
-      </c>
-      <c r="B45" t="s">
-        <v>200</v>
       </c>
       <c r="C45" t="s">
         <v>34</v>
@@ -3019,24 +3436,33 @@
         <v>36</v>
       </c>
       <c r="F45" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G45" t="s">
         <v>66</v>
       </c>
       <c r="H45" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="I45" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J45" t="s">
+        <v>236</v>
+      </c>
+      <c r="K45" s="71" t="s">
+        <v>235</v>
+      </c>
+      <c r="L45" s="71"/>
+      <c r="M45" s="71"/>
+      <c r="N45" s="71"/>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" s="64" t="s">
+        <v>202</v>
+      </c>
+      <c r="B46" t="s">
         <v>203</v>
-      </c>
-      <c r="B46" t="s">
-        <v>204</v>
       </c>
       <c r="C46" t="s">
         <v>34</v>
@@ -3051,7 +3477,7 @@
         <v>37</v>
       </c>
       <c r="G46" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="H46" t="s">
         <v>39</v>
@@ -3059,45 +3485,63 @@
       <c r="I46" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J46" t="s">
+        <v>233</v>
+      </c>
+      <c r="K46" s="71" t="s">
+        <v>239</v>
+      </c>
+      <c r="L46" s="71"/>
+      <c r="M46" s="71"/>
+      <c r="N46" s="71"/>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" s="64" t="s">
+        <v>205</v>
+      </c>
+      <c r="B47" t="s">
         <v>206</v>
       </c>
-      <c r="B47" t="s">
-        <v>207</v>
-      </c>
       <c r="C47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D47" t="s">
         <v>35</v>
       </c>
       <c r="E47" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F47" t="s">
         <v>61</v>
       </c>
       <c r="G47" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H47" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="I47" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J47" t="s">
+        <v>234</v>
+      </c>
+      <c r="K47" s="71" t="s">
+        <v>144</v>
+      </c>
+      <c r="L47" s="71"/>
+      <c r="M47" s="71"/>
+      <c r="N47" s="71"/>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" s="64" t="s">
+        <v>208</v>
+      </c>
+      <c r="B48" t="s">
         <v>209</v>
       </c>
-      <c r="B48" t="s">
-        <v>210</v>
-      </c>
       <c r="C48" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D48" t="s">
         <v>35</v>
@@ -3106,27 +3550,36 @@
         <v>1</v>
       </c>
       <c r="F48" t="s">
+        <v>116</v>
+      </c>
+      <c r="G48" t="s">
         <v>117</v>
       </c>
-      <c r="G48" t="s">
-        <v>118</v>
-      </c>
       <c r="H48" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I48" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J48" t="s">
+        <v>233</v>
+      </c>
+      <c r="K48" s="71" t="s">
+        <v>99</v>
+      </c>
+      <c r="L48" s="71"/>
+      <c r="M48" s="71"/>
+      <c r="N48" s="71"/>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="64" t="s">
+        <v>210</v>
+      </c>
+      <c r="B49" t="s">
         <v>211</v>
       </c>
-      <c r="B49" t="s">
-        <v>212</v>
-      </c>
       <c r="C49" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D49" t="s">
         <v>35</v>
@@ -3141,18 +3594,27 @@
         <v>56</v>
       </c>
       <c r="H49" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I49" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J49" t="s">
+        <v>234</v>
+      </c>
+      <c r="K49" s="71" t="s">
+        <v>99</v>
+      </c>
+      <c r="L49" s="71"/>
+      <c r="M49" s="71"/>
+      <c r="N49" s="71"/>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" s="64" t="s">
+        <v>212</v>
+      </c>
+      <c r="B50" t="s">
         <v>213</v>
-      </c>
-      <c r="B50" t="s">
-        <v>214</v>
       </c>
       <c r="C50" t="s">
         <v>34</v>
@@ -3175,13 +3637,22 @@
       <c r="I50" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J50" t="s">
+        <v>233</v>
+      </c>
+      <c r="K50" s="71" t="s">
+        <v>242</v>
+      </c>
+      <c r="L50" s="71"/>
+      <c r="M50" s="71"/>
+      <c r="N50" s="71"/>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" s="64" t="s">
+        <v>214</v>
+      </c>
+      <c r="B51" t="s">
         <v>215</v>
-      </c>
-      <c r="B51" t="s">
-        <v>216</v>
       </c>
       <c r="C51" t="s">
         <v>34</v>
@@ -3190,27 +3661,36 @@
         <v>35</v>
       </c>
       <c r="E51" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F51" t="s">
         <v>49</v>
       </c>
       <c r="G51" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="H51" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I51" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J51" t="s">
+        <v>234</v>
+      </c>
+      <c r="K51" s="71" t="s">
+        <v>240</v>
+      </c>
+      <c r="L51" s="71"/>
+      <c r="M51" s="71"/>
+      <c r="N51" s="71"/>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52" s="64" t="s">
+        <v>217</v>
+      </c>
+      <c r="B52" t="s">
         <v>218</v>
-      </c>
-      <c r="B52" t="s">
-        <v>219</v>
       </c>
       <c r="C52" t="s">
         <v>34</v>
@@ -3228,18 +3708,27 @@
         <v>62</v>
       </c>
       <c r="H52" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="I52" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J52" t="s">
+        <v>233</v>
+      </c>
+      <c r="K52" s="71" t="s">
+        <v>242</v>
+      </c>
+      <c r="L52" s="71"/>
+      <c r="M52" s="71"/>
+      <c r="N52" s="71"/>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" s="64" t="s">
+        <v>220</v>
+      </c>
+      <c r="B53" t="s">
         <v>221</v>
-      </c>
-      <c r="B53" t="s">
-        <v>222</v>
       </c>
       <c r="C53" t="s">
         <v>34</v>
@@ -3251,7 +3740,7 @@
         <v>36</v>
       </c>
       <c r="F53" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G53" t="s">
         <v>66</v>
@@ -3262,13 +3751,22 @@
       <c r="I53" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J53" t="s">
+        <v>234</v>
+      </c>
+      <c r="K53" s="71" t="s">
+        <v>241</v>
+      </c>
+      <c r="L53" s="71"/>
+      <c r="M53" s="71"/>
+      <c r="N53" s="71"/>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="64" t="s">
+        <v>222</v>
+      </c>
+      <c r="B54" t="s">
         <v>223</v>
-      </c>
-      <c r="B54" t="s">
-        <v>224</v>
       </c>
       <c r="C54" t="s">
         <v>34</v>
@@ -3286,21 +3784,30 @@
         <v>82</v>
       </c>
       <c r="H54" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I54" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J54" t="s">
+        <v>67</v>
+      </c>
+      <c r="K54" s="71" t="s">
+        <v>245</v>
+      </c>
+      <c r="L54" s="71"/>
+      <c r="M54" s="71"/>
+      <c r="N54" s="71"/>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" s="64" t="s">
+        <v>224</v>
+      </c>
+      <c r="B55" t="s">
         <v>225</v>
       </c>
-      <c r="B55" t="s">
-        <v>226</v>
-      </c>
       <c r="C55" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D55" t="s">
         <v>35</v>
@@ -3309,36 +3816,45 @@
         <v>1</v>
       </c>
       <c r="F55" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G55" t="s">
         <v>88</v>
       </c>
       <c r="H55" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I55" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J55" t="s">
+        <v>234</v>
+      </c>
+      <c r="K55" s="71" t="s">
+        <v>99</v>
+      </c>
+      <c r="L55" s="71"/>
+      <c r="M55" s="71"/>
+      <c r="N55" s="71"/>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" s="64" t="s">
+        <v>226</v>
+      </c>
+      <c r="B56" t="s">
         <v>227</v>
-      </c>
-      <c r="B56" t="s">
-        <v>228</v>
       </c>
       <c r="C56" t="s">
         <v>34</v>
       </c>
       <c r="D56" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E56" t="s">
         <v>1</v>
       </c>
       <c r="F56" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G56" t="s">
         <v>50</v>
@@ -3349,8 +3865,17 @@
       <c r="I56" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J56" t="s">
+        <v>67</v>
+      </c>
+      <c r="K56" s="71" t="s">
+        <v>245</v>
+      </c>
+      <c r="L56" s="71"/>
+      <c r="M56" s="71"/>
+      <c r="N56" s="71"/>
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A57" s="64"/>
       <c r="B57" s="64"/>
       <c r="C57" s="64"/>
@@ -3360,13 +3885,11 @@
       <c r="G57" s="64"/>
       <c r="H57" s="64"/>
       <c r="I57" s="64"/>
+      <c r="L57" s="71"/>
+      <c r="M57" s="71"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:I51" xr:uid="{EF946802-625C-4B02-AEB9-0F5333A1D5C8}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:I56">
-      <sortCondition ref="A2:A51"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="B2:K2" xr:uid="{EF946802-625C-4B02-AEB9-0F5333A1D5C8}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -7807,17 +8330,17 @@
   <sheetData>
     <row r="2" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B2" s="24" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="3" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="5" spans="2:2" x14ac:dyDescent="0.25">
@@ -7827,7 +8350,7 @@
     </row>
     <row r="6" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.25">
@@ -7837,7 +8360,7 @@
     </row>
     <row r="8" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>

</xml_diff>